<commit_message>
SkyG Speed 90: printable F2 (wall-grown bridges, G-code audited), rear wing screw at LE + 58, 30 % lightning infill
</commit_message>
<xml_diff>
--- a/c6/downloads/C6/SkyG-Speed-90-BOM.xlsx
+++ b/c6/downloads/C6/SkyG-Speed-90-BOM.xlsx
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Z-bend in the servo arm (holes drilled to 1.3 mm), 90° L-bend through the printed horn, keeper on the end</t>
+          <t>Z-bend in the servo arm (hole drilled 1.1 mm, reamed to 1.2 mm), 90° L-bend through the printed horn (reamed the same), keeper on the end</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Z-bend pliers, 1.3 mm drill, small flat file</t>
+          <t>Z-bend pliers, 1.1 mm drill, 1.2 mm drill (as a hand reamer), small flat file</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Pliers for the 90° L-bends; 1.3 mm drill for the servo-arm holes; flat file for the 0.3 mm flats</t>
+          <t>Pliers for the 90° L-bends; servo-arm and horn holes drilled 1.1 mm then reamed by hand with the 1.2 mm bit (zero play); flat file for the 0.3 mm flats</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Tools: servo arms drilled to 1.3 mm, flats on the stabilator shafts (under the printed horns) and the torque rods</t>
+          <t>Tools: servo-arm and horn holes reamed to 1.2 mm, flats on the stabilator shafts (under the printed horns) and the torque rods</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Nylon countersunk screw M3 x 8</t>
+          <t>Nylon countersunk screw M3 x 12</t>
         </is>
       </c>
       <c r="D52" s="7" t="n">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>M3x8 nylon countersunk screw</t>
+          <t>M3x12 nylon countersunk screw</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>Wing mount, rear screw (x = wing LE + 84)</t>
+          <t>Wing mount, rear screw (x = wing LE + 58, ahead of the aileron horns)</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>A 12 mm screw here reaches the aileron servo arm (found with the screws modelled in the assembly)</t>
+          <t>2026-10-07: moved from LE + 84 so its nut bridge can grow from the side walls on a pointed-arch lead-in (DFAM A2l; at LE + 84 the lead-in ran through the aileron horns' sweep). The wing is 7.4 mm thick there: 12 mm reaches through the nut</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>15T 3.9-4 mm spline arms: two-sided (aileron) with holes at 4.3 mm, one-sided (tail) with a hole at 6.7 mm; C6: holes drilled to 1.3 mm for the 1.2 mm Z-bends</t>
+          <t>15T 3.9-4 mm spline arms: two-sided (aileron) with holes at 4.3 mm, one-sided (tail) with a hole at 6.7 mm; C6: holes drilled 1.1 mm and reamed to 1.2 mm for the 1.2 mm Z-bends (no play)</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
@@ -3369,17 +3369,17 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3395,17 +3395,17 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3421,17 +3421,17 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.39</v>
+        <v>0.41</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3577,17 +3577,17 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.7</v>
+        <v>0.79</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3603,17 +3603,17 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>6.1</v>
+        <v>6.7</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>0.64</v>
+        <v>0.7</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3629,17 +3629,17 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>1.89</v>
+        <v>1.93</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3655,17 +3655,17 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>20.6</v>
+        <v>21.7</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>2.08</v>
+        <v>2.18</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3681,17 +3681,17 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.99</v>
+        <v>1.04</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>0 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3733,17 +3733,17 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -3759,10 +3759,10 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>15.4</v>
+        <v>16.3</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>2.58</v>
+        <v>2.6</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
@@ -3788,7 +3788,7 @@
         <v>16.3</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>2.59</v>
+        <v>2.6</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
@@ -3811,10 +3811,10 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>0.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E22" s="7" t="n">
         <v>1</v>
@@ -3837,10 +3837,10 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>1</v>
@@ -3941,17 +3941,17 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>5.4</v>
+        <v>4.5</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>15 %</t>
+          <t>30 %</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 107.5 g, 15.7 h of printing.</t>
+          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 109.5 g, 15.9 h of printing.</t>
         </is>
       </c>
     </row>

</xml_diff>